<commit_message>
Complete Executive Overview Page(1)
</commit_message>
<xml_diff>
--- a/dashboard/Complete_Dashboard_Planning_Matrix.xlsx
+++ b/dashboard/Complete_Dashboard_Planning_Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\fabric-olist-ecommerce-analytics\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{12311B28-AF71-46D3-B2AF-EA5DAA516FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{21EABC4A-5B27-4320-95B1-88F399069A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard Summary" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="208">
   <si>
     <t>Page</t>
   </si>
@@ -631,13 +631,34 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>+--------------------------------------------------------------------------------------+</t>
+  </si>
+  <si>
+    <t>| KPI Cards: GMV | Orders | Customers | Avg Order | Delivery | Review               |</t>
+  </si>
+  <si>
+    <t>| Top Categories                                  | Payment Method Distribution                       |</t>
+  </si>
+  <si>
+    <t>| Monthly Trend                                  | Orders by Status                                                 |</t>
+  </si>
+  <si>
+    <t>| Revenue by State                              | Delivery Performance                                       |</t>
+  </si>
+  <si>
+    <t>| Navigation                                                                                                                              |</t>
+  </si>
+  <si>
+    <t>| Title | Last Refresh | Year | Month | State                                                                    |</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -656,6 +677,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Cambria"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -678,10 +705,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1142,45 +1170,74 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="53.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C3" s="3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C4" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C5" s="3" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="C6" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C7" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="C8" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>102</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C10" s="3" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>